<commit_message>
carga masiva de productos
</commit_message>
<xml_diff>
--- a/PedidosBarrio/plantillas/plantilla_producto.xlsx
+++ b/PedidosBarrio/plantillas/plantilla_producto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\proyectos\Tienda\backend\PedidosBarrioBackend\PedidosBarrio\plantillas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EC58905A-B5A4-4C2B-A61C-50661166BD18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A3261E87-9242-4B9B-B50C-D3C760F5D212}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="46">
   <si>
     <t>NombreProducto*</t>
   </si>
@@ -36,24 +36,9 @@
     <t>Visible</t>
   </si>
   <si>
-    <t>NombrePresentacion</t>
-  </si>
-  <si>
-    <t>DescripcionOpcion</t>
-  </si>
-  <si>
-    <t>Polo Básico</t>
-  </si>
-  <si>
-    <t>Polo de algodón</t>
-  </si>
-  <si>
     <t>Talla</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>M</t>
   </si>
   <si>
@@ -120,9 +105,6 @@
     <t>Codigo</t>
   </si>
   <si>
-    <t>abc-de-55</t>
-  </si>
-  <si>
     <t>abc-de-66</t>
   </si>
   <si>
@@ -133,6 +115,51 @@
   </si>
   <si>
     <t>L</t>
+  </si>
+  <si>
+    <t>Presentacion</t>
+  </si>
+  <si>
+    <t>NombrePresentacion1</t>
+  </si>
+  <si>
+    <t>DescripcionOpcion1</t>
+  </si>
+  <si>
+    <t>NombrePresentacion2</t>
+  </si>
+  <si>
+    <t>DescripcionOpcion2</t>
+  </si>
+  <si>
+    <t>NombrePresentacion3</t>
+  </si>
+  <si>
+    <t>DescripcionOpcion3</t>
+  </si>
+  <si>
+    <t>pruebas</t>
+  </si>
+  <si>
+    <t>Camisa oversize talla M, color rojo</t>
+  </si>
+  <si>
+    <t>Color</t>
+  </si>
+  <si>
+    <t>Rojo</t>
+  </si>
+  <si>
+    <t>Camisa oversize talla M, color verde</t>
+  </si>
+  <si>
+    <t>Verde</t>
+  </si>
+  <si>
+    <t>Camisa oversize talla L, color rojo</t>
+  </si>
+  <si>
+    <t>Camisa oversize talla L, color verde</t>
   </si>
 </sst>
 </file>
@@ -160,7 +187,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="9">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -191,6 +218,24 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -204,18 +249,27 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -530,7 +584,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:M7"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="2" width="12.6640625" customWidth="1"/>
@@ -541,152 +595,218 @@
     <col min="7" max="7" width="12.109375" customWidth="1"/>
     <col min="8" max="8" width="22.21875" customWidth="1"/>
     <col min="9" max="9" width="24.6640625" customWidth="1"/>
+    <col min="10" max="10" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-    </row>
-    <row r="2" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="4" t="s">
+      <c r="H1" s="4"/>
+      <c r="I1" s="4"/>
+      <c r="J1" s="4"/>
+      <c r="K1" s="4"/>
+      <c r="L1" s="4"/>
+      <c r="M1" s="4"/>
+    </row>
+    <row r="2" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="H2" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="I2" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="J2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="K2" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="L2" s="7" t="s">
+        <v>36</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" t="s">
         <v>29</v>
       </c>
-      <c r="H2" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="I2" s="4" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>32</v>
-      </c>
-      <c r="B3" t="s">
-        <v>22</v>
-      </c>
-      <c r="C3" t="s">
-        <v>6</v>
-      </c>
       <c r="D3" t="s">
-        <v>7</v>
+        <v>39</v>
       </c>
       <c r="E3">
         <v>5</v>
       </c>
       <c r="F3" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G3">
-        <v>30.5</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+        <v>80</v>
+      </c>
+      <c r="H3" t="s">
+        <v>4</v>
+      </c>
+      <c r="I3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J3" t="s">
+        <v>40</v>
+      </c>
+      <c r="K3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B4" t="s">
+        <v>38</v>
+      </c>
+      <c r="C4" t="s">
+        <v>29</v>
+      </c>
+      <c r="D4" t="s">
+        <v>42</v>
+      </c>
+      <c r="E4">
+        <v>5</v>
+      </c>
+      <c r="F4" t="s">
         <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>35</v>
-      </c>
-      <c r="E4">
-        <v>0</v>
-      </c>
-      <c r="F4" t="s">
-        <v>28</v>
       </c>
       <c r="G4">
         <v>80</v>
       </c>
-      <c r="H4" t="s">
-        <v>8</v>
-      </c>
       <c r="I4" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+        <v>5</v>
+      </c>
+      <c r="K4" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>38</v>
       </c>
       <c r="C5" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>35</v>
+        <v>44</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
       </c>
       <c r="F5" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="G5">
         <v>85</v>
       </c>
-      <c r="H5" t="s">
-        <v>8</v>
-      </c>
       <c r="I5" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+        <v>30</v>
+      </c>
+      <c r="K5" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>38</v>
       </c>
       <c r="C6" t="s">
-        <v>11</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>12</v>
+        <v>45</v>
+      </c>
+      <c r="E6">
+        <v>1</v>
       </c>
       <c r="F6" t="s">
+        <v>23</v>
+      </c>
+      <c r="G6">
+        <v>85</v>
+      </c>
+      <c r="I6" t="s">
+        <v>30</v>
+      </c>
+      <c r="K6" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="A7" t="s">
         <v>28</v>
       </c>
-      <c r="G6">
+      <c r="B7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C7" t="s">
+        <v>6</v>
+      </c>
+      <c r="D7" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" t="s">
+        <v>23</v>
+      </c>
+      <c r="G7">
         <v>60</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="G1:I1"/>
+    <mergeCell ref="G1:M1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
   <extLst>
@@ -696,7 +816,7 @@
           <x14:formula1>
             <xm:f>Categoria!$A$2:$A$8</xm:f>
           </x14:formula1>
-          <xm:sqref>B3:B1048576</xm:sqref>
+          <xm:sqref>B8:B1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -714,42 +834,42 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
     </row>
   </sheetData>
@@ -770,37 +890,37 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" spans="1:1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>